<commit_message>
Add geschaeftsreise: ICE Fahrkarte Augsburg-Mannheim
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
@@ -417,22 +417,21 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M8"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="23" customWidth="1" min="1" max="1"/>
     <col width="34" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="22" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
     <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="13" customWidth="1" min="11" max="11"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -453,50 +452,45 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Lieferant</t>
+          <t>Datum</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Datum</t>
+          <t>Einzelkosten</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Einzelkosten</t>
+          <t>Währung</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Währung</t>
+          <t>Ort</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>Ort</t>
+          <t>Land</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Land</t>
+          <t>Reisebeginn</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Reisebeginn</t>
+          <t>Reiseende</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Reiseende</t>
+          <t>Kategorie</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>Kategorie</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Bemerkung</t>
         </is>
@@ -505,7 +499,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>ICE-690-Ticket.md</t>
+          <t>ICE-690-Fahrkarte.md</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -518,30 +512,30 @@
           <t>Bahnticket</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>– nicht angegeben –</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+      <c r="D2" t="inlineStr"/>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>26,99</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>26,99</t>
+          <t>€</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>€</t>
+          <t>Mannheim</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>Mannheim</t>
+          <t>Deutschland</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>Deutschland</t>
+          <t>30.01.2026</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -551,15 +545,10 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>30.01.2026</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
           <t>Reise</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr"/>
+      <c r="L2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
@@ -586,7 +575,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>26.99</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add geschaeftsreise: ICE Fahrkarte Augsburg - Mannheim
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
@@ -417,11 +417,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="23" customWidth="1" min="1" max="1"/>
-    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="36" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="8" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
@@ -512,7 +512,6 @@
           <t>Bahnticket</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>26,99</t>
@@ -548,8 +547,9 @@
           <t>Reise</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr"/>
-    </row>
+    </row>
+    <row r="3"/>
+    <row r="4"/>
     <row r="5">
       <c r="A5" s="1" t="inlineStr">
         <is>
@@ -561,6 +561,7 @@
         <v/>
       </c>
     </row>
+    <row r="6"/>
     <row r="7">
       <c r="A7" s="1" t="inlineStr">
         <is>
@@ -575,6 +576,88 @@
         </is>
       </c>
       <c r="B8" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>ICE-690-Ticket.md</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>ICE Fahrkarte Augsburg - Mannheim</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>26,99</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>€</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Mannheim</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>30.01.2026</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>31.01.2026</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Gesamtkosten</t>
+        </is>
+      </c>
+      <c r="B12">
+        <f>SUM(F2:F9)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add geschaeftsreise: Bahnfahrkarte Mannheim - Augsburg
</commit_message>
<xml_diff>
--- a/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
+++ b/Inbox/Geschaeftsreise/2026/Q1/2026-01-30_Mannheim/Reiseübersicht.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Übersicht" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$L$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Übersicht'!$A$1:$L$13</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -19,8 +19,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="2">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="165" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="164" formatCode="DD.MM.YYYY"/>
+    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -77,7 +77,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -88,7 +88,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -104,6 +104,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -472,7 +475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L8"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -567,7 +570,7 @@
           <t>Bahnticket</t>
         </is>
       </c>
-      <c r="D2" s="4" t="n">
+      <c r="D2" s="10" t="n">
         <v>46052</v>
       </c>
       <c r="E2" s="5" t="n">
@@ -588,10 +591,10 @@
           <t>Deutschland</t>
         </is>
       </c>
-      <c r="I2" s="4" t="n">
+      <c r="I2" s="10" t="n">
         <v>46052</v>
       </c>
-      <c r="J2" s="4" t="n">
+      <c r="J2" s="10" t="n">
         <v>46053</v>
       </c>
       <c r="K2" s="3" t="inlineStr">
@@ -602,99 +605,124 @@
       <c r="L2" s="3" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="n"/>
-      <c r="B3" s="6" t="n"/>
-      <c r="C3" s="6" t="n"/>
-      <c r="D3" s="6" t="n"/>
-      <c r="E3" s="6" t="n"/>
-      <c r="F3" s="6" t="n"/>
-      <c r="G3" s="6" t="n"/>
-      <c r="H3" s="6" t="n"/>
-      <c r="I3" s="6" t="n"/>
-      <c r="J3" s="6" t="n"/>
-      <c r="K3" s="6" t="n"/>
-      <c r="L3" s="6" t="n"/>
+      <c r="A3" s="3" t="n"/>
+      <c r="B3" s="3" t="n"/>
+      <c r="C3" s="3" t="n"/>
+      <c r="D3" s="3" t="n"/>
+      <c r="E3" s="3" t="n"/>
+      <c r="F3" s="3" t="n"/>
+      <c r="G3" s="3" t="n"/>
+      <c r="H3" s="3" t="n"/>
+      <c r="I3" s="3" t="n"/>
+      <c r="J3" s="3" t="n"/>
+      <c r="K3" s="3" t="n"/>
+      <c r="L3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="n"/>
-      <c r="B4" s="6" t="n"/>
-      <c r="C4" s="6" t="n"/>
-      <c r="D4" s="6" t="n"/>
-      <c r="E4" s="6" t="n"/>
-      <c r="F4" s="6" t="n"/>
-      <c r="G4" s="6" t="n"/>
-      <c r="H4" s="6" t="n"/>
-      <c r="I4" s="6" t="n"/>
-      <c r="J4" s="6" t="n"/>
-      <c r="K4" s="6" t="n"/>
-      <c r="L4" s="6" t="n"/>
+      <c r="A4" s="3" t="n"/>
+      <c r="B4" s="3" t="n"/>
+      <c r="C4" s="3" t="n"/>
+      <c r="D4" s="3" t="n"/>
+      <c r="E4" s="3" t="n"/>
+      <c r="F4" s="3" t="n"/>
+      <c r="G4" s="3" t="n"/>
+      <c r="H4" s="3" t="n"/>
+      <c r="I4" s="3" t="n"/>
+      <c r="J4" s="3" t="n"/>
+      <c r="K4" s="3" t="n"/>
+      <c r="L4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="7" t="inlineStr">
-        <is>
-          <t>Gesamtkosten</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="n"/>
-      <c r="C5" s="6" t="n"/>
-      <c r="D5" s="6" t="n"/>
-      <c r="E5" s="8">
-        <f>SUM(E2:E2)</f>
+      <c r="A5" s="3" t="n"/>
+      <c r="B5" s="3" t="n"/>
+      <c r="C5" s="3" t="n"/>
+      <c r="D5" s="3" t="n"/>
+      <c r="E5" s="3" t="n"/>
+      <c r="F5" s="3" t="n"/>
+      <c r="G5" s="3" t="n"/>
+      <c r="H5" s="3" t="n"/>
+      <c r="I5" s="3" t="n"/>
+      <c r="J5" s="3" t="n"/>
+      <c r="K5" s="3" t="n"/>
+      <c r="L5" s="3" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="n"/>
+      <c r="C6" s="3" t="n"/>
+      <c r="D6" s="3" t="n"/>
+      <c r="E6" s="5">
+        <f>SUMIF(C2:C2,"Bahnticket",E2:E2)</f>
         <v/>
       </c>
-      <c r="F5" s="6" t="n"/>
-      <c r="G5" s="6" t="n"/>
-      <c r="H5" s="6" t="n"/>
-      <c r="I5" s="6" t="n"/>
-      <c r="J5" s="6" t="n"/>
-      <c r="K5" s="6" t="n"/>
-      <c r="L5" s="6" t="n"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
+      <c r="F6" s="3" t="n"/>
+      <c r="G6" s="3" t="n"/>
+      <c r="H6" s="3" t="n"/>
+      <c r="I6" s="3" t="n"/>
+      <c r="J6" s="3" t="n"/>
+      <c r="K6" s="3" t="n"/>
+      <c r="L6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
-        <is>
-          <t>Kosten nach Dokumentart</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="n"/>
-      <c r="C7" s="6" t="n"/>
-      <c r="D7" s="6" t="n"/>
-      <c r="E7" s="6" t="n"/>
-      <c r="F7" s="6" t="n"/>
-      <c r="G7" s="6" t="n"/>
-      <c r="H7" s="6" t="n"/>
-      <c r="I7" s="6" t="n"/>
-      <c r="J7" s="6" t="n"/>
-      <c r="K7" s="6" t="n"/>
-      <c r="L7" s="6" t="n"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ICE-919-Ticket.md</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Bahnfahrkarte Mannheim - Augsburg</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="D7" s="10" t="n">
+        <v>46052</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>23.99</v>
+      </c>
+      <c r="F7" s="3" t="inlineStr">
+        <is>
+          <t>EUR</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
+        <is>
+          <t>Mannheim</t>
+        </is>
+      </c>
+      <c r="H7" s="3" t="inlineStr">
+        <is>
+          <t>Deutschland</t>
+        </is>
+      </c>
+      <c r="I7" s="10" t="n">
+        <v>46052</v>
+      </c>
+      <c r="J7" s="10" t="n">
+        <v>46055</v>
+      </c>
+      <c r="K7" s="3" t="inlineStr">
+        <is>
+          <t>Reise</t>
+        </is>
+      </c>
+      <c r="L7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>Bahnticket</t>
-        </is>
-      </c>
+      <c r="A8" s="6" t="n"/>
       <c r="B8" s="6" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
-      <c r="E8" s="9">
-        <f>SUMIF(C2:C2,"Bahnticket",E2:E2)</f>
-        <v/>
-      </c>
+      <c r="E8" s="6" t="n"/>
       <c r="F8" s="6" t="n"/>
       <c r="G8" s="6" t="n"/>
       <c r="H8" s="6" t="n"/>
@@ -703,10 +731,99 @@
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="n"/>
     </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+      <c r="F9" s="6" t="n"/>
+      <c r="G9" s="6" t="n"/>
+      <c r="H9" s="6" t="n"/>
+      <c r="I9" s="6" t="n"/>
+      <c r="J9" s="6" t="n"/>
+      <c r="K9" s="6" t="n"/>
+      <c r="L9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Gesamtkosten</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="8">
+        <f>SUM(E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F10" s="6" t="n"/>
+      <c r="G10" s="6" t="n"/>
+      <c r="H10" s="6" t="n"/>
+      <c r="I10" s="6" t="n"/>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="n"/>
+      <c r="L10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+      <c r="F11" s="6" t="n"/>
+      <c r="G11" s="6" t="n"/>
+      <c r="H11" s="6" t="n"/>
+      <c r="I11" s="6" t="n"/>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="n"/>
+      <c r="L11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Kosten nach Dokumentart</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+      <c r="F12" s="6" t="n"/>
+      <c r="G12" s="6" t="n"/>
+      <c r="H12" s="6" t="n"/>
+      <c r="I12" s="6" t="n"/>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="n"/>
+      <c r="L12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="inlineStr">
+        <is>
+          <t>Bahnticket</t>
+        </is>
+      </c>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="9">
+        <f>SUMIF(C2:C7,"Bahnticket",E2:E7)</f>
+        <v/>
+      </c>
+      <c r="F13" s="6" t="n"/>
+      <c r="G13" s="6" t="n"/>
+      <c r="H13" s="6" t="n"/>
+      <c r="I13" s="6" t="n"/>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="n"/>
+      <c r="L13" s="6" t="n"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:L8"/>
+  <autoFilter ref="A1:L13"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A2" r:id="rId1"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId2"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>

</xml_diff>